<commit_message>
new script combining ana's misclass scripts
</commit_message>
<xml_diff>
--- a/misclass_dir/Output/COTA_misclassified_patterns_colored.xlsx
+++ b/misclass_dir/Output/COTA_misclassified_patterns_colored.xlsx
@@ -8250,7 +8250,7 @@
       </c>
       <c r="K34" s="17" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies + Proteasome inhibitors (Not in provided Fiona's category list)</t>
+          <t>Monoclonal antibodies + Proteasome inhibitors</t>
         </is>
       </c>
       <c r="L34" s="17" t="inlineStr">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>IMiDs + Steroids + Other non-chemotherapy (Not in provided Fiona's category list)</t>
+          <t>IMiDs + Steroids + Other non-chemotherapy</t>
         </is>
       </c>
       <c r="L48" s="11" t="inlineStr">
@@ -11896,7 +11896,7 @@
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>IMiDs + Steroids + Other non-chemotherapy (Not in provided Fiona's category list)</t>
+          <t>IMiDs + Steroids + Other non-chemotherapy</t>
         </is>
       </c>
       <c r="L50" s="13" t="inlineStr">
@@ -16942,7 +16942,7 @@
       </c>
       <c r="K72" s="15" t="inlineStr">
         <is>
-          <t>CAR-T + Transplant (Not in provided Fiona's category list)</t>
+          <t>CAR-T + Transplant</t>
         </is>
       </c>
       <c r="L72" s="15" t="inlineStr">
@@ -18389,7 +18389,7 @@
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>CAR-T + Transplant (Not in provided Fiona's category list)</t>
+          <t>CAR-T + Transplant</t>
         </is>
       </c>
       <c r="B23" s="21" t="inlineStr">
@@ -18605,7 +18605,7 @@
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
         <is>
-          <t>IMiDs + Steroids + Other non-chemotherapy (Not in provided Fiona's category list)</t>
+          <t>IMiDs + Steroids + Other non-chemotherapy</t>
         </is>
       </c>
       <c r="B35" s="21" t="inlineStr">
@@ -18623,7 +18623,7 @@
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
         <is>
-          <t>IMiDs + Steroids + Other non-chemotherapy (Not in provided Fiona's category list)</t>
+          <t>IMiDs + Steroids + Other non-chemotherapy</t>
         </is>
       </c>
       <c r="B36" s="21" t="inlineStr">
@@ -18659,7 +18659,7 @@
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies + Proteasome inhibitors (Not in provided Fiona's category list)</t>
+          <t>Monoclonal antibodies + Proteasome inhibitors</t>
         </is>
       </c>
       <c r="B38" s="21" t="inlineStr">
@@ -26678,7 +26678,7 @@
       </c>
       <c r="K35" s="21" t="inlineStr">
         <is>
-          <t>IMiDs + Steroids + Other non-chemotherapy (Not in provided Fiona's category list)</t>
+          <t>IMiDs + Steroids + Other non-chemotherapy</t>
         </is>
       </c>
       <c r="L35" s="21" t="inlineStr">
@@ -32559,7 +32559,7 @@
       </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies + Proteasome inhibitors (Not in provided Fiona's category list)</t>
+          <t>Monoclonal antibodies + Proteasome inhibitors</t>
         </is>
       </c>
       <c r="L10" s="21" t="inlineStr">
@@ -33941,7 +33941,7 @@
       </c>
       <c r="K16" s="21" t="inlineStr">
         <is>
-          <t>IMiDs + Steroids + Other non-chemotherapy (Not in provided Fiona's category list)</t>
+          <t>IMiDs + Steroids + Other non-chemotherapy</t>
         </is>
       </c>
       <c r="L16" s="21" t="inlineStr">
@@ -36281,7 +36281,7 @@
       </c>
       <c r="K26" s="21" t="inlineStr">
         <is>
-          <t>CAR-T + Transplant (Not in provided Fiona's category list)</t>
+          <t>CAR-T + Transplant</t>
         </is>
       </c>
       <c r="L26" s="21" t="inlineStr">

</xml_diff>